<commit_message>
feat: add Excel upload functionality and PDF line items table template for project bill of quantities
</commit_message>
<xml_diff>
--- a/app/BillOfQuantities/data/Project set-up Template.xlsx
+++ b/app/BillOfQuantities/data/Project set-up Template.xlsx
@@ -7733,7 +7733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O1000"/>
+  <dimension ref="A1:S1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="29.7109375" bestFit="1" customWidth="1" style="31" min="1" max="1"/>
@@ -7788,17 +7788,17 @@
       </c>
       <c r="H1" s="182" t="inlineStr">
         <is>
-          <t>Contract Quantity</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="I1" s="183" t="inlineStr">
         <is>
-          <t>Contract Rate</t>
+          <t>Rate</t>
         </is>
       </c>
       <c r="J1" s="184" t="inlineStr">
         <is>
-          <t>Contract Amount</t>
+          <t>Amount</t>
         </is>
       </c>
     </row>
@@ -22955,12 +22955,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B3:C6"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="108.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="15.75" customHeight="1" thickBot="1"/>
     <row r="3" ht="15.75" customHeight="1" thickBot="1">
       <c r="C3" s="178" t="inlineStr">
@@ -23005,6 +23006,9 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23016,7 +23020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O571"/>
+  <dimension ref="A1:S571"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="29.7109375" bestFit="1" customWidth="1" style="31" min="1" max="1"/>
@@ -23071,17 +23075,17 @@
       </c>
       <c r="H1" s="182" t="inlineStr">
         <is>
-          <t>Contract Quantity</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="I1" s="183" t="inlineStr">
         <is>
-          <t>Contract Rate</t>
+          <t>Rate</t>
         </is>
       </c>
       <c r="J1" s="184" t="inlineStr">
         <is>
-          <t>Contract Amount</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="K1" s="3" t="n">

</xml_diff>

<commit_message>
feat: add Project set-up Template.xlsx to BillOfQuantities data directory
</commit_message>
<xml_diff>
--- a/app/BillOfQuantities/data/Project set-up Template.xlsx
+++ b/app/BillOfQuantities/data/Project set-up Template.xlsx
@@ -7733,7 +7733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O1000"/>
+  <dimension ref="A1:S1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="29.7109375" bestFit="1" customWidth="1" style="31" min="1" max="1"/>
@@ -7788,17 +7788,17 @@
       </c>
       <c r="H1" s="182" t="inlineStr">
         <is>
-          <t>Contract Quantity</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="I1" s="183" t="inlineStr">
         <is>
-          <t>Contract Rate</t>
+          <t>Rate</t>
         </is>
       </c>
       <c r="J1" s="184" t="inlineStr">
         <is>
-          <t>Contract Amount</t>
+          <t>Amount</t>
         </is>
       </c>
     </row>
@@ -22955,12 +22955,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B3:C6"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="108.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="15.75" customHeight="1" thickBot="1"/>
     <row r="3" ht="15.75" customHeight="1" thickBot="1">
       <c r="C3" s="178" t="inlineStr">
@@ -23005,6 +23006,9 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23016,7 +23020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O571"/>
+  <dimension ref="A1:S571"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="29.7109375" bestFit="1" customWidth="1" style="31" min="1" max="1"/>
@@ -23071,17 +23075,17 @@
       </c>
       <c r="H1" s="182" t="inlineStr">
         <is>
-          <t>Contract Quantity</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="I1" s="183" t="inlineStr">
         <is>
-          <t>Contract Rate</t>
+          <t>Rate</t>
         </is>
       </c>
       <c r="J1" s="184" t="inlineStr">
         <is>
-          <t>Contract Amount</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="K1" s="3" t="n">

</xml_diff>